<commit_message>
Actualización automática: datos al 2026-09-13
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>249041205.24</v>
+        <v>249096025.57</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>689334696.9299999</v>
+        <v>689496019.98</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>249041205.24</v>
+        <v>249096025.57</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689334696.9299999</v>
+        <v>689496019.98</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.001309</v>
+        <v>0.001439</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.00271</v>
+        <v>0.002944</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5985,6 +5985,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46277</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18723551</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.00013</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>249096025.57</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1053.09013095</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>689496019.98</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1241.24667396</v>
@@ -49462,7 +49480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
         </is>
       </c>
     </row>
@@ -49805,7 +49823,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18708163</v>
+        <v>1.18723551</v>
       </c>
     </row>
     <row r="5">
@@ -49925,7 +49943,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1052.84373691</v>
+        <v>1053.09013095</v>
       </c>
     </row>
     <row r="6">
@@ -50322,7 +50340,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
         </is>
       </c>
     </row>
@@ -50665,7 +50683,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>249041205.24</v>
+        <v>249096025.57</v>
       </c>
     </row>
     <row r="5">
@@ -50785,7 +50803,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>689334696.9299999</v>
+        <v>689496019.98</v>
       </c>
     </row>
     <row r="6">
@@ -51151,7 +51169,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-13 (actualización 2026-09-12).</t>
+          <t>datos al 2026-09-13 (actualización 2026-09-13).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-14
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>249096025.57</v>
+        <v>249118122.33</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>689496019.98</v>
+        <v>689657900.01</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>249096025.57</v>
+        <v>249118122.33</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689496019.98</v>
+        <v>689657900.01</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.001439</v>
+        <v>0.001569</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.002944</v>
+        <v>0.00318</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5944,6 +5944,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46278</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18739018</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.00013</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>249118122.33</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1053.3373757</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>689657900.01</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1241.42837718</v>
@@ -49480,7 +49498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -49823,7 +49841,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18723551</v>
+        <v>1.18739018</v>
       </c>
     </row>
     <row r="5">
@@ -49943,7 +49961,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1053.09013095</v>
+        <v>1053.3373757</v>
       </c>
     </row>
     <row r="6">
@@ -50340,7 +50358,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-13)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-13 (actualización 2026-09-14)</t>
         </is>
       </c>
     </row>
@@ -50683,7 +50701,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>249096025.57</v>
+        <v>249118122.33</v>
       </c>
     </row>
     <row r="5">
@@ -50803,7 +50821,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>689496019.98</v>
+        <v>689657900.01</v>
       </c>
     </row>
     <row r="6">
@@ -51169,7 +51187,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-13 (actualización 2026-09-13).</t>
+          <t>datos al 2026-09-13 (actualización 2026-09-14).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-16
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>245981620.76</v>
+        <v>246074001.98</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>689818848.76</v>
+        <v>689979878.25</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>245981620.76</v>
+        <v>246074001.98</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689818848.76</v>
+        <v>689979878.25</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.001695</v>
+        <v>0.001826</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.003414</v>
+        <v>0.003648</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5944,6 +5944,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46280</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18769446</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>246074001.98</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1053.82914373</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>689979878.25</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1241.78842587</v>
@@ -49598,7 +49616,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16)</t>
         </is>
       </c>
     </row>
@@ -49941,7 +49959,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18753906</v>
+        <v>1.18769446</v>
       </c>
     </row>
     <row r="5">
@@ -50061,7 +50079,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1053.58319805</v>
+        <v>1053.82914373</v>
       </c>
     </row>
     <row r="6">
@@ -50458,7 +50476,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-15 (actualización 2026-09-16)</t>
         </is>
       </c>
     </row>
@@ -50801,7 +50819,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>245981620.76</v>
+        <v>246074001.98</v>
       </c>
     </row>
     <row r="5">
@@ -50921,7 +50939,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>689818848.76</v>
+        <v>689979878.25</v>
       </c>
     </row>
     <row r="6">
@@ -51287,7 +51305,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-15 (actualización 2026-09-15).</t>
+          <t>datos al 2026-09-15 (actualización 2026-09-16).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-20
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>238089786.38</v>
+        <v>238248152.41</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>690463172.8099999</v>
+        <v>690624380.02</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>238089786.38</v>
+        <v>238248152.41</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>690463172.8099999</v>
+        <v>690624380.02</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.002212</v>
+        <v>0.002344</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.004351</v>
+        <v>0.004586</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5985,6 +5985,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46284</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18830839</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>238248152.41</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1054.81351265</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>690624380.02</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1242.43478648</v>
@@ -49875,7 +49893,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
         </is>
       </c>
     </row>
@@ -50218,7 +50236,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18815211</v>
+        <v>1.18830839</v>
       </c>
     </row>
     <row r="5">
@@ -50338,7 +50356,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1054.56729554</v>
+        <v>1054.81351265</v>
       </c>
     </row>
     <row r="6">
@@ -50735,7 +50753,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
         </is>
       </c>
     </row>
@@ -51078,7 +51096,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>238089786.38</v>
+        <v>238248152.41</v>
       </c>
     </row>
     <row r="5">
@@ -51198,7 +51216,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>690463172.8099999</v>
+        <v>690624380.02</v>
       </c>
     </row>
     <row r="6">
@@ -51564,7 +51582,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-20 (actualización 2026-09-19).</t>
+          <t>datos al 2026-09-20 (actualización 2026-09-20).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-21
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>238248152.41</v>
+        <v>238279970.22</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>690624380.02</v>
+        <v>690786281.12</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>238248152.41</v>
+        <v>238279970.22</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>690624380.02</v>
+        <v>690786281.12</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.002344</v>
+        <v>0.002475</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.004586</v>
+        <v>0.004821</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5944,6 +5944,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46285</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18846448</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>238279970.22</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1055.06078957</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>690786281.12</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1242.58916097</v>
@@ -49893,7 +49911,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21)</t>
         </is>
       </c>
     </row>
@@ -50236,7 +50254,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18830839</v>
+        <v>1.18846448</v>
       </c>
     </row>
     <row r="5">
@@ -50356,7 +50374,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1054.81351265</v>
+        <v>1055.06078957</v>
       </c>
     </row>
     <row r="6">
@@ -50753,7 +50771,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-20)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-20 (actualización 2026-09-21)</t>
         </is>
       </c>
     </row>
@@ -51096,7 +51114,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>238248152.41</v>
+        <v>238279970.22</v>
       </c>
     </row>
     <row r="5">
@@ -51216,7 +51234,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>690624380.02</v>
+        <v>690786281.12</v>
       </c>
     </row>
     <row r="6">
@@ -51582,7 +51600,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-20 (actualización 2026-09-20).</t>
+          <t>datos al 2026-09-20 (actualización 2026-09-21).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-27
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>227005416.09</v>
+        <v>227145263.77</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>686799310.97</v>
+        <v>686960396.1900001</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>227005416.09</v>
+        <v>227145263.77</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>686799310.97</v>
+        <v>686960396.1900001</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.003143</v>
+        <v>0.003276</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>-0.0009779999999999999</v>
+        <v>-0.000744</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5985,6 +5985,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46291</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18941373</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>227145263.77</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1049.21738868</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>686960396.1900001</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1243.54194648</v>
@@ -50288,7 +50306,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
         </is>
       </c>
     </row>
@@ -50631,7 +50649,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18925557</v>
+        <v>1.18941373</v>
       </c>
     </row>
     <row r="5">
@@ -50751,7 +50769,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1048.97135788</v>
+        <v>1049.21738868</v>
       </c>
     </row>
     <row r="6">
@@ -51148,7 +51166,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
         </is>
       </c>
     </row>
@@ -51491,7 +51509,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>227005416.09</v>
+        <v>227145263.77</v>
       </c>
     </row>
     <row r="5">
@@ -51611,7 +51629,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>686799310.97</v>
+        <v>686960396.1900001</v>
       </c>
     </row>
     <row r="6">
@@ -51977,7 +51995,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-27 (actualización 2026-09-26).</t>
+          <t>datos al 2026-09-27 (actualización 2026-09-27).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-28
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>227145263.77</v>
+        <v>227150042.02</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>686960396.1900001</v>
+        <v>687122005.55</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>227145263.77</v>
+        <v>227150042.02</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>686960396.1900001</v>
+        <v>687122005.55</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.003276</v>
+        <v>0.003409</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>-0.000744</v>
+        <v>-0.000509</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5944,6 +5944,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46292</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18957179</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>227150042.02</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1049.46422001</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>687122005.55</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1243.76205507</v>
@@ -50306,7 +50324,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -50649,7 +50667,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18941373</v>
+        <v>1.18957179</v>
       </c>
     </row>
     <row r="5">
@@ -50769,7 +50787,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1049.21738868</v>
+        <v>1049.46422001</v>
       </c>
     </row>
     <row r="6">
@@ -51166,7 +51184,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-27)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-27 (actualización 2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -51509,7 +51527,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>227145263.77</v>
+        <v>227150042.02</v>
       </c>
     </row>
     <row r="5">
@@ -51629,7 +51647,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>686960396.1900001</v>
+        <v>687122005.55</v>
       </c>
     </row>
     <row r="6">
@@ -51995,7 +52013,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-27 (actualización 2026-09-27).</t>
+          <t>datos al 2026-09-27 (actualización 2026-09-28).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-10-04
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AQ4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AQ5</f>
@@ -3190,7 +3190,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ2" t="n">
-        <v>240982080.91</v>
+        <v>241109958.39</v>
       </c>
     </row>
     <row r="3">
@@ -3308,7 +3308,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ3" t="n">
-        <v>687914868.0599999</v>
+        <v>688076212.9400001</v>
       </c>
     </row>
     <row r="4">
@@ -3589,7 +3589,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>240982080.91</v>
+        <v>241109958.39</v>
       </c>
     </row>
     <row r="12">
@@ -3608,7 +3608,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>687914868.0599999</v>
+        <v>688076212.9400001</v>
       </c>
     </row>
     <row r="13">
@@ -4010,7 +4010,7 @@
         <v>0.003787</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.000272</v>
+        <v>0.000402</v>
       </c>
     </row>
     <row r="21">
@@ -4128,7 +4128,7 @@
         <v>0.000176</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.000468</v>
+        <v>0.000702</v>
       </c>
     </row>
     <row r="22">
@@ -4390,7 +4390,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6061,6 +6061,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46298</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.19049876</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>241109958.39</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1050.92161259</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>688076212.9400001</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1244.85815926</v>
@@ -50778,7 +50796,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -51129,7 +51147,7 @@
         <v>1.19001996</v>
       </c>
       <c r="AQ4" s="24" t="n">
-        <v>1.19034313</v>
+        <v>1.19049876</v>
       </c>
     </row>
     <row r="5">
@@ -51252,7 +51270,7 @@
         <v>1050.18404187</v>
       </c>
       <c r="AQ5" s="24" t="n">
-        <v>1050.6751852</v>
+        <v>1050.92161259</v>
       </c>
     </row>
     <row r="6">
@@ -51662,7 +51680,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -52013,7 +52031,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ4" s="25" t="n">
-        <v>240982080.91</v>
+        <v>241109958.39</v>
       </c>
     </row>
     <row r="5">
@@ -52136,7 +52154,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ5" s="25" t="n">
-        <v>687914868.0599999</v>
+        <v>688076212.9400001</v>
       </c>
     </row>
     <row r="6">
@@ -52514,7 +52532,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-10-04 (actualización 2026-10-03).</t>
+          <t>datos al 2026-10-04 (actualización 2026-10-04).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-10-05
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AQ4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AQ5</f>
@@ -3190,7 +3190,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ2" t="n">
-        <v>241109958.39</v>
+        <v>241120859.78</v>
       </c>
     </row>
     <row r="3">
@@ -3308,7 +3308,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ3" t="n">
-        <v>688076212.9400001</v>
+        <v>688237549.92</v>
       </c>
     </row>
     <row r="4">
@@ -3589,7 +3589,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>241109958.39</v>
+        <v>241120859.78</v>
       </c>
     </row>
     <row r="12">
@@ -3608,7 +3608,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>688076212.9400001</v>
+        <v>688237549.92</v>
       </c>
     </row>
     <row r="13">
@@ -4010,7 +4010,7 @@
         <v>0.003787</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.000402</v>
+        <v>0.0005330000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -4128,7 +4128,7 @@
         <v>0.000176</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.000702</v>
+        <v>0.000937</v>
       </c>
     </row>
     <row r="22">
@@ -4390,7 +4390,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6020,6 +6020,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46299</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.1906543</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>241120859.78</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1051.16802791</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>688237549.92</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1245.00372336</v>
@@ -50796,7 +50814,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05)</t>
         </is>
       </c>
     </row>
@@ -51147,7 +51165,7 @@
         <v>1.19001996</v>
       </c>
       <c r="AQ4" s="24" t="n">
-        <v>1.19049876</v>
+        <v>1.1906543</v>
       </c>
     </row>
     <row r="5">
@@ -51270,7 +51288,7 @@
         <v>1050.18404187</v>
       </c>
       <c r="AQ5" s="24" t="n">
-        <v>1050.92161259</v>
+        <v>1051.16802791</v>
       </c>
     </row>
     <row r="6">
@@ -51680,7 +51698,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-04 (actualización 2026-10-05)</t>
         </is>
       </c>
     </row>
@@ -52031,7 +52049,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ4" s="25" t="n">
-        <v>241109958.39</v>
+        <v>241120859.78</v>
       </c>
     </row>
     <row r="5">
@@ -52154,7 +52172,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ5" s="25" t="n">
-        <v>688076212.9400001</v>
+        <v>688237549.92</v>
       </c>
     </row>
     <row r="6">
@@ -52532,7 +52550,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-10-04 (actualización 2026-10-04).</t>
+          <t>datos al 2026-10-04 (actualización 2026-10-05).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-10-11
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AQ4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AQ5</f>
@@ -3190,7 +3190,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ2" t="n">
-        <v>258885996.09</v>
+        <v>259948863.18</v>
       </c>
     </row>
     <row r="3">
@@ -3308,7 +3308,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ3" t="n">
-        <v>689043277.22</v>
+        <v>689204672.71</v>
       </c>
     </row>
     <row r="4">
@@ -3589,7 +3589,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>258885996.09</v>
+        <v>259948863.18</v>
       </c>
     </row>
     <row r="12">
@@ -3608,7 +3608,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689043277.22</v>
+        <v>689204672.71</v>
       </c>
     </row>
     <row r="13">
@@ -4010,7 +4010,7 @@
         <v>0.003787</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.001189</v>
+        <v>0.001318</v>
       </c>
     </row>
     <row r="21">
@@ -4128,7 +4128,7 @@
         <v>0.000176</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.002109</v>
+        <v>0.002343</v>
       </c>
     </row>
     <row r="22">
@@ -4390,7 +4390,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6061,6 +6061,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46305</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.19158847</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000129</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>259948863.18</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1052.64514661</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>689204672.71</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1245.85466691</v>
@@ -51191,7 +51209,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -51542,7 +51560,7 @@
         <v>1.19001996</v>
       </c>
       <c r="AQ4" s="24" t="n">
-        <v>1.19143477</v>
+        <v>1.19158847</v>
       </c>
     </row>
     <row r="5">
@@ -51665,7 +51683,7 @@
         <v>1050.18404187</v>
       </c>
       <c r="AQ5" s="24" t="n">
-        <v>1052.39864193</v>
+        <v>1052.64514661</v>
       </c>
     </row>
     <row r="6">
@@ -52075,7 +52093,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-10)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -52426,7 +52444,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ4" s="25" t="n">
-        <v>258885996.09</v>
+        <v>259948863.18</v>
       </c>
     </row>
     <row r="5">
@@ -52549,7 +52567,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ5" s="25" t="n">
-        <v>689043277.22</v>
+        <v>689204672.71</v>
       </c>
     </row>
     <row r="6">
@@ -52927,7 +52945,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-10-11 (actualización 2026-10-10).</t>
+          <t>datos al 2026-10-11 (actualización 2026-10-11).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-10-12
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AQ4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AQ5</f>
@@ -3190,7 +3190,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ2" t="n">
-        <v>259948863.18</v>
+        <v>260138330.17</v>
       </c>
     </row>
     <row r="3">
@@ -3308,7 +3308,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ3" t="n">
-        <v>689204672.71</v>
+        <v>689365403.9400001</v>
       </c>
     </row>
     <row r="4">
@@ -3589,7 +3589,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>259948863.18</v>
+        <v>260138330.17</v>
       </c>
     </row>
     <row r="12">
@@ -3608,7 +3608,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689204672.71</v>
+        <v>689365403.9400001</v>
       </c>
     </row>
     <row r="13">
@@ -4010,7 +4010,7 @@
         <v>0.003787</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.001318</v>
+        <v>0.001449</v>
       </c>
     </row>
     <row r="21">
@@ -4128,7 +4128,7 @@
         <v>0.000176</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.002343</v>
+        <v>0.002577</v>
       </c>
     </row>
     <row r="22">
@@ -4390,7 +4390,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6020,6 +6020,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46306</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.1917438</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.00013</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>260138330.17</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1052.89063676</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>689365403.9400001</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1245.99461404</v>
@@ -51209,7 +51227,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -51560,7 +51578,7 @@
         <v>1.19001996</v>
       </c>
       <c r="AQ4" s="24" t="n">
-        <v>1.19158847</v>
+        <v>1.1917438</v>
       </c>
     </row>
     <row r="5">
@@ -51683,7 +51701,7 @@
         <v>1050.18404187</v>
       </c>
       <c r="AQ5" s="24" t="n">
-        <v>1052.64514661</v>
+        <v>1052.89063676</v>
       </c>
     </row>
     <row r="6">
@@ -52093,7 +52111,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-10-11 (actualización 2026-10-12)</t>
         </is>
       </c>
     </row>
@@ -52444,7 +52462,7 @@
         <v>230374844.97</v>
       </c>
       <c r="AQ4" s="25" t="n">
-        <v>259948863.18</v>
+        <v>260138330.17</v>
       </c>
     </row>
     <row r="5">
@@ -52567,7 +52585,7 @@
         <v>687593298.84</v>
       </c>
       <c r="AQ5" s="25" t="n">
-        <v>689204672.71</v>
+        <v>689365403.9400001</v>
       </c>
     </row>
     <row r="6">
@@ -52945,7 +52963,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-10-11 (actualización 2026-10-11).</t>
+          <t>datos al 2026-10-11 (actualización 2026-10-12).</t>
         </is>
       </c>
     </row>

</xml_diff>